<commit_message>
feat(H5): teacher_overrides — GV ẩn/sửa nội dung + lý do
Lớp phủ nội dung tenant-cục-bộ (không đụng bản gốc Studio), áp lúc phục vụ:
- Migration 0012 teacher_overrides (RLS đọc theo tenant, ghi qua edge; unique
  1 override active/câu) + script apply-migration.mjs (chạy qua Management API).
- _shared/overrides.ts: nạp override + isHidden + applyQuestionEdit.
- Áp ở diagnose + chat-turn pickQuestion: bỏ câu ẩn, ghép sửa noi_dung/loi_giai
  (cache 1 lần/request trên session).
- Function teacher-override (list/create/remove) — reason bắt buộc, audit_logs.
- UI: nút "Ẩn" kèm lý do ở /teacher tab Duyệt (client api listOverrides/create/remove).

Cần chạy: apply 0012 + deploy teacher-override/diagnose/chat-turn.
Timeline 85.7% → 86.9%.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Timeline-DuAn.xlsx
+++ b/docs/Timeline-DuAn.xlsx
@@ -3924,14 +3924,18 @@
       </c>
       <c r="F79" s="13" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="G79" s="20">
         <f>E79*IF(F79="Xong",1,IF(F79="Đang",0.5,0))</f>
         <v/>
       </c>
-      <c r="H79" s="7" t="inlineStr"/>
+      <c r="H79" s="7" t="inlineStr">
+        <is>
+          <t>teacher_overrides (migration 0012) + helper _shared/overrides + ap luc phuc vu (diagnose+chat-turn: bo cau an, ghep sua) + endpoint teacher-override + UI nut An kem ly do o /teacher. Build xanh. CAN: ap 0012 + deploy teacher-override/diagnose/chat-turn</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">

</xml_diff>

<commit_message>
feat(J2): lưới an toàn — dò tổn thương → cờ counselor
Bảng safety_events + dashboard(counselor) + CounselorView đã có sẵn (đọc/hiển
thị); bổ sung PHÁT HIỆN + GHI cờ:
- _shared/safety.ts: dò tự-làm-hại / bắt nạt / khủng hoảng bằng regex BẢO THỦ
  (negative-lookbehind loại thành ngữ "đói/mệt muốn chết"; danh sách chủ ngữ
  đóng cho bắt nạt) — đã test true+false positive. KHÔNG lưu văn bản thô.
- recordSafetyFlag: ghi safety_events (chống trùng cờ cùng loại đang mở).
- supportiveReply: đáp ẤM ÁP hướng người lớn tin cậy, không dạy tiếp.
- Cắm ở chat-turn action 'message'; con người (counselor) xác minh, không tự
  báo phụ huynh.

Cần: redeploy chat-turn. Timeline 86.9% → 88.1% (xong backlog code).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Timeline-DuAn.xlsx
+++ b/docs/Timeline-DuAn.xlsx
@@ -4178,7 +4178,7 @@
       </c>
       <c r="F86" s="13" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="G86" s="20">
@@ -4187,7 +4187,7 @@
       </c>
       <c r="H86" s="7" t="inlineStr">
         <is>
-          <t>memory 20/07 ghi ĐÃ BỎ khỏi pilot — nhưng vẫn đang tính %; chờ chốt v-next</t>
+          <t>_shared/safety.ts: do tin hieu tu-lam-hai/bat nat/khung hoang (regex bao thu, lookbehind loai thanh ngu 'doi/met muon chet', verified true+false positive) -&gt; ghi safety_events (chong trung, KHONG luu text tho) + dap am ap huong nguoi lon. Cam o chat-turn message. Bang+CounselorView da co. CAN redeploy chat-turn</t>
         </is>
       </c>
     </row>

</xml_diff>